<commit_message>
Move codon transforms to structure rows
</commit_message>
<xml_diff>
--- a/supporting_material/experiments/example-dual-display/example-dual-display-extended.xlsx
+++ b/supporting_material/experiments/example-dual-display/example-dual-display-extended.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-10660" yWindow="-32740" windowWidth="32500" windowHeight="25020" tabRatio="500" firstSheet="0" activeTab="10" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="experiment" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reaction_graph" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -70,12 +70,6 @@
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -499,27 +493,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -528,55 +522,55 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -585,69 +579,69 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -911,7 +905,8 @@
   <cols>
     <col width="10.1640625" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="17" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
-    <col width="10.83203125" customWidth="1" style="7" min="3" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="3" max="3"/>
+    <col width="10.83203125" customWidth="1" style="7" min="4" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -934,7 +929,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>campaign</t>
+          <t>campaign-extended</t>
         </is>
       </c>
     </row>
@@ -984,7 +979,8 @@
   <cols>
     <col width="7.5" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="108.5" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
-    <col width="10.6640625" customWidth="1" style="7" min="3" max="16384"/>
+    <col width="10.6640625" customWidth="1" style="7" min="3" max="3"/>
+    <col width="10.6640625" customWidth="1" style="7" min="4" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3912,14 +3908,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col width="5.83203125" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="12.83203125" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
     <col width="14" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
     <col width="6.1640625" bestFit="1" customWidth="1" style="7" min="4" max="4"/>
-    <col width="10.83203125" customWidth="1" style="7" min="5" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="5" max="5"/>
+    <col width="10.83203125" customWidth="1" style="7" min="6" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
@@ -3948,6 +3945,16 @@
           <t>strand</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reverse</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>complement</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="67" t="inlineStr">
@@ -3967,6 +3974,12 @@
         <v>0</v>
       </c>
       <c r="E2" s="69" t="n"/>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
@@ -3986,6 +3999,12 @@
         <v>0</v>
       </c>
       <c r="E3" s="50" t="n"/>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -4009,6 +4028,12 @@
           <t>A</t>
         </is>
       </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -4028,6 +4053,12 @@
         <v>0</v>
       </c>
       <c r="E5" s="50" t="n"/>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -4051,6 +4082,12 @@
           <t>A</t>
         </is>
       </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -4070,6 +4107,12 @@
         <v>0</v>
       </c>
       <c r="E7" s="50" t="n"/>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -4093,6 +4136,12 @@
           <t>B</t>
         </is>
       </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
@@ -4112,6 +4161,12 @@
         <v>0</v>
       </c>
       <c r="E9" s="50" t="n"/>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4135,6 +4190,12 @@
           <t>B</t>
         </is>
       </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -4154,6 +4215,12 @@
         <v>0</v>
       </c>
       <c r="E11" s="50" t="n"/>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" thickBot="1">
       <c r="A12" s="16" t="inlineStr">
@@ -4173,6 +4240,12 @@
         <v>0</v>
       </c>
       <c r="E12" s="37" t="n"/>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4278,7 +4351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M612"/>
+  <dimension ref="A1:K612"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="54.1640625" defaultRowHeight="16"/>
   <cols>
     <col width="7.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4315,16 +4388,6 @@
         </is>
       </c>
       <c r="H1" s="39" t="n"/>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>reverse</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>complement</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="63" t="inlineStr">
@@ -4356,12 +4419,6 @@
       <c r="I2" s="38" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="63" t="inlineStr">
@@ -4393,12 +4450,6 @@
       <c r="I3" s="38" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
@@ -4430,12 +4481,6 @@
       <c r="I4" s="38" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="63" t="inlineStr">
@@ -4467,12 +4512,6 @@
       <c r="I5" s="38" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
-      <c r="L5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="63" t="inlineStr">
@@ -4504,12 +4543,6 @@
       <c r="I6" s="38" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="H7" s="38" t="n"/>
@@ -4517,153 +4550,6 @@
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
     <row r="155">
       <c r="J155" s="2" t="n"/>
     </row>
@@ -6565,7 +6451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="7.1640625" bestFit="1" customWidth="1" style="52" min="1" max="1"/>
@@ -6573,7 +6459,8 @@
     <col width="9.33203125" bestFit="1" customWidth="1" style="52" min="3" max="3"/>
     <col width="6.83203125" bestFit="1" customWidth="1" style="52" min="4" max="4"/>
     <col width="8.33203125" bestFit="1" customWidth="1" style="52" min="5" max="5"/>
-    <col width="12.83203125" customWidth="1" style="52" min="6" max="16384"/>
+    <col width="12.83203125" customWidth="1" style="52" min="6" max="6"/>
+    <col width="12.83203125" customWidth="1" style="52" min="7" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
@@ -6602,18 +6489,8 @@
           <t>product</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>reverse</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>complement</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
           <t>ATGCGT</t>
@@ -6639,14 +6516,8 @@
           <t>product_2</t>
         </is>
       </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="53" t="inlineStr">
         <is>
           <t>CAATAG</t>
@@ -6671,12 +6542,6 @@
         <is>
           <t>product_2</t>
         </is>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6699,7 +6564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M612"/>
+  <dimension ref="A1:K612"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="54.1640625" defaultRowHeight="16"/>
   <cols>
     <col width="7.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6736,16 +6601,6 @@
         </is>
       </c>
       <c r="H1" s="39" t="n"/>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>reverse</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>complement</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="63" t="inlineStr">
@@ -6777,12 +6632,6 @@
       <c r="I2" s="38" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
-      <c r="L2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="63" t="inlineStr">
@@ -6814,12 +6663,6 @@
       <c r="I3" s="38" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
@@ -6851,12 +6694,6 @@
       <c r="I4" s="38" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="63" t="inlineStr">
@@ -6888,12 +6725,6 @@
       <c r="I5" s="38" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="63" t="inlineStr">
@@ -6925,12 +6756,6 @@
       <c r="I6" s="38" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="H7" s="38" t="n"/>
@@ -6938,153 +6763,6 @@
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
     <row r="155">
       <c r="J155" s="2" t="n"/>
     </row>
@@ -8986,7 +8664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="7.1640625" bestFit="1" customWidth="1" style="52" min="1" max="1"/>
@@ -8994,7 +8672,8 @@
     <col width="9.33203125" bestFit="1" customWidth="1" style="52" min="3" max="3"/>
     <col width="6.83203125" bestFit="1" customWidth="1" style="52" min="4" max="4"/>
     <col width="8.33203125" bestFit="1" customWidth="1" style="52" min="5" max="5"/>
-    <col width="12.83203125" customWidth="1" style="52" min="6" max="16384"/>
+    <col width="12.83203125" customWidth="1" style="52" min="6" max="6"/>
+    <col width="12.83203125" customWidth="1" style="52" min="7" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
@@ -9023,18 +8702,8 @@
           <t>product</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>reverse</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>complement</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
           <t>TAGGAC</t>
@@ -9060,14 +8729,8 @@
           <t>product_4</t>
         </is>
       </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="53" t="inlineStr">
         <is>
           <t>CTGTAT</t>
@@ -9092,12 +8755,6 @@
         <is>
           <t>product_4</t>
         </is>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9125,7 +8782,8 @@
   <cols>
     <col width="9.5" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="30.1640625" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
-    <col width="10.6640625" customWidth="1" style="7" min="3" max="16384"/>
+    <col width="10.6640625" customWidth="1" style="7" min="3" max="3"/>
+    <col width="10.6640625" customWidth="1" style="7" min="4" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>